<commit_message>
summary table for strat 1254 obs and its simulation performance
</commit_message>
<xml_diff>
--- a/data/september strat simulation/latest(for stakeholder)/strat1254_obs/result_20261007_164841(VN_strat1254_obs_07Oct).xlsx
+++ b/data/september strat simulation/latest(for stakeholder)/strat1254_obs/result_20261007_164841(VN_strat1254_obs_07Oct).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wei.kc\Desktop\Adhoc\03 Sept 2026\data\september strat simulation\latest(for stakeholder)\strat1254_obs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B80855E9-F8C8-4A46-9333-47413C9E552C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF7B608B-032E-4E19-9923-7E4BC380267F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2568" uniqueCount="402">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2575" uniqueCount="408">
   <si>
     <t>traceid</t>
   </si>
@@ -1360,30 +1360,15 @@
     <t>Strategy Observation</t>
   </si>
   <si>
-    <t>True Positives (Accounts)</t>
-  </si>
-  <si>
-    <t>False Positives (Accounts)</t>
-  </si>
-  <si>
     <t>Account Precision</t>
   </si>
   <si>
     <t>Order level</t>
   </si>
   <si>
-    <t>Hit Rate (%)</t>
-  </si>
-  <si>
     <t>Hit Count (Orders)</t>
   </si>
   <si>
-    <t>True Positives (Orders)</t>
-  </si>
-  <si>
-    <t>False Positives (Orders)</t>
-  </si>
-  <si>
     <t>Order Precision</t>
   </si>
   <si>
@@ -1394,17 +1379,51 @@
   </si>
   <si>
     <t>0.00253%</t>
+  </si>
+  <si>
+    <t>Hit Rate (Accounts)</t>
+  </si>
+  <si>
+    <t>0.00064%</t>
+  </si>
+  <si>
+    <t>Hit Count (Accounts)</t>
+  </si>
+  <si>
+    <t>True Positive (Accounts)</t>
+  </si>
+  <si>
+    <t>False Positive (Accounts)</t>
+  </si>
+  <si>
+    <t>True Positive (Orders)</t>
+  </si>
+  <si>
+    <t>False Positive (Orders)</t>
+  </si>
+  <si>
+    <t>Hit Rate (Orders)</t>
+  </si>
+  <si>
+    <t>Simulation</t>
+  </si>
+  <si>
+    <t>81.82% (279 / 341)</t>
+  </si>
+  <si>
+    <t>84.44% (17879 / 21173)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
     <numFmt numFmtId="170" formatCode="0.00000"/>
+    <numFmt numFmtId="180" formatCode="0.00000%"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -1434,8 +1453,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1448,8 +1474,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="8">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -1562,13 +1594,80 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFDEE0E3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFDEE0E3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFDEE0E3"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDEE0E3"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1588,13 +1687,29 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="3" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -13770,10 +13885,10 @@
     <col min="8" max="8" width="18" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15.44140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.109375" customWidth="1"/>
     <col min="14" max="14" width="21" customWidth="1"/>
     <col min="15" max="15" width="16.109375" customWidth="1"/>
-    <col min="16" max="16" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.3">
@@ -14432,106 +14547,157 @@
         <v>379</v>
       </c>
     </row>
-    <row r="17" spans="14:15" x14ac:dyDescent="0.3">
+    <row r="17" spans="14:16" x14ac:dyDescent="0.3">
       <c r="N17" s="12" t="s">
         <v>387</v>
       </c>
       <c r="O17" s="12"/>
     </row>
-    <row r="18" spans="14:15" x14ac:dyDescent="0.3">
-      <c r="N18" s="13" t="s">
+    <row r="18" spans="14:16" x14ac:dyDescent="0.3">
+      <c r="N18" s="22" t="s">
         <v>388</v>
       </c>
-      <c r="O18" s="14" t="s">
+      <c r="O18" s="23" t="s">
         <v>389</v>
       </c>
-    </row>
-    <row r="19" spans="14:15" x14ac:dyDescent="0.3">
-      <c r="N19" s="15" t="s">
+      <c r="P18" s="22" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="19" spans="14:16" x14ac:dyDescent="0.3">
+      <c r="N19" s="17" t="s">
+        <v>397</v>
+      </c>
+      <c r="O19" s="18" t="s">
+        <v>398</v>
+      </c>
+      <c r="P19" s="26">
+        <v>5.4258841724890165E-4</v>
+      </c>
+    </row>
+    <row r="20" spans="14:16" x14ac:dyDescent="0.3">
+      <c r="N20" s="20" t="s">
+        <v>399</v>
+      </c>
+      <c r="O20" s="17">
+        <v>15</v>
+      </c>
+      <c r="P20" s="17">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="21" spans="14:16" x14ac:dyDescent="0.3">
+      <c r="N21" s="21" t="s">
+        <v>400</v>
+      </c>
+      <c r="O21" s="21">
+        <v>12</v>
+      </c>
+      <c r="P21" s="16">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="22" spans="14:16" x14ac:dyDescent="0.3">
+      <c r="N22" s="21" t="s">
+        <v>401</v>
+      </c>
+      <c r="O22" s="21">
+        <v>3</v>
+      </c>
+      <c r="P22" s="13">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="23" spans="14:16" x14ac:dyDescent="0.3">
+      <c r="N23" s="21" t="s">
         <v>390</v>
       </c>
-      <c r="O19" s="16">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="20" spans="14:15" x14ac:dyDescent="0.3">
-      <c r="N20" s="15" t="s">
+      <c r="O23" s="21" t="s">
+        <v>394</v>
+      </c>
+      <c r="P23" s="14" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="24" spans="14:16" x14ac:dyDescent="0.3">
+      <c r="N24" s="19"/>
+      <c r="O24" s="19"/>
+      <c r="P24" s="27"/>
+    </row>
+    <row r="25" spans="14:16" x14ac:dyDescent="0.3">
+      <c r="N25" s="12" t="s">
         <v>391</v>
       </c>
-      <c r="O20" s="16">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21" spans="14:15" x14ac:dyDescent="0.3">
-      <c r="N21" s="15" t="s">
+      <c r="O25" s="12"/>
+      <c r="P25" s="27"/>
+    </row>
+    <row r="26" spans="14:16" x14ac:dyDescent="0.3">
+      <c r="N26" s="24" t="s">
+        <v>388</v>
+      </c>
+      <c r="O26" s="25" t="s">
+        <v>389</v>
+      </c>
+      <c r="P26" s="24" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="27" spans="14:16" x14ac:dyDescent="0.3">
+      <c r="N27" s="13" t="s">
+        <v>404</v>
+      </c>
+      <c r="O27" s="15" t="s">
+        <v>396</v>
+      </c>
+      <c r="P27" s="28">
+        <v>2.4479794255497693E-3</v>
+      </c>
+    </row>
+    <row r="28" spans="14:16" x14ac:dyDescent="0.3">
+      <c r="N28" s="13" t="s">
         <v>392</v>
       </c>
-      <c r="O21" s="16" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="22" spans="14:15" x14ac:dyDescent="0.3">
-      <c r="N22" s="12"/>
-      <c r="O22" s="12"/>
-    </row>
-    <row r="23" spans="14:15" x14ac:dyDescent="0.3">
-      <c r="N23" s="12" t="s">
-        <v>393</v>
-      </c>
-      <c r="O23" s="12"/>
-    </row>
-    <row r="24" spans="14:15" x14ac:dyDescent="0.3">
-      <c r="N24" s="13" t="s">
-        <v>388</v>
-      </c>
-      <c r="O24" s="14" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="25" spans="14:15" x14ac:dyDescent="0.3">
-      <c r="N25" s="15" t="s">
-        <v>394</v>
-      </c>
-      <c r="O25" s="17" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="26" spans="14:15" x14ac:dyDescent="0.3">
-      <c r="N26" s="15" t="s">
-        <v>395</v>
-      </c>
-      <c r="O26" s="16">
+      <c r="O28" s="14">
         <v>201</v>
       </c>
-    </row>
-    <row r="27" spans="14:15" x14ac:dyDescent="0.3">
-      <c r="N27" s="15" t="s">
-        <v>396</v>
-      </c>
-      <c r="O27" s="16">
+      <c r="P28" s="29">
+        <v>21173</v>
+      </c>
+    </row>
+    <row r="29" spans="14:16" x14ac:dyDescent="0.3">
+      <c r="N29" s="13" t="s">
+        <v>402</v>
+      </c>
+      <c r="O29" s="14">
         <f>SUMIF($K$2:$K$16,N2,$F$2:$F$16)</f>
         <v>172</v>
       </c>
-    </row>
-    <row r="28" spans="14:15" x14ac:dyDescent="0.3">
-      <c r="N28" s="15" t="s">
-        <v>397</v>
-      </c>
-      <c r="O28" s="16">
+      <c r="P29" s="29">
+        <v>17879</v>
+      </c>
+    </row>
+    <row r="30" spans="14:16" x14ac:dyDescent="0.3">
+      <c r="N30" s="13" t="s">
+        <v>403</v>
+      </c>
+      <c r="O30" s="14">
         <f>SUMIF($K$2:$K$16,N3,$F$2:$F$16)</f>
         <v>29</v>
       </c>
-    </row>
-    <row r="29" spans="14:15" x14ac:dyDescent="0.3">
-      <c r="N29" s="15" t="s">
-        <v>398</v>
-      </c>
-      <c r="O29" s="16" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="31" spans="14:15" x14ac:dyDescent="0.3">
-      <c r="O31" s="10"/>
+      <c r="P30" s="29">
+        <v>3294</v>
+      </c>
+    </row>
+    <row r="31" spans="14:16" x14ac:dyDescent="0.3">
+      <c r="N31" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="O31" s="14" t="s">
+        <v>395</v>
+      </c>
+      <c r="P31" s="14" t="s">
+        <v>407</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>